<commit_message>
commit latest review on 27thMarch
</commit_message>
<xml_diff>
--- a/testdata/demodata.xlsx
+++ b/testdata/demodata.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\DHANUNJAYA\DHANUNJAYA LAPTOP\Automation Training\API Automation\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\DHANUNJAYA\DHANUNJAYA LAPTOP\Automation Training\API Automation\feedback\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13593D67-2DD8-411D-A610-BC5040B3AE62}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{9D4B404B-DCC0-4346-A4A9-AD0EC4123E55}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7425" xr2:uid="{0B2E8F83-0EBC-4F7F-BFBA-398DDD676471}"/>
   </bookViews>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="41">
   <si>
     <t>TestCases</t>
   </si>
@@ -96,6 +96,60 @@
   </si>
   <si>
     <t>Test</t>
+  </si>
+  <si>
+    <t>AddPlace</t>
+  </si>
+  <si>
+    <t>EcomOrder</t>
+  </si>
+  <si>
+    <t>Laptop</t>
+  </si>
+  <si>
+    <t>fashion</t>
+  </si>
+  <si>
+    <t>shirts</t>
+  </si>
+  <si>
+    <t>Lenova</t>
+  </si>
+  <si>
+    <t>India</t>
+  </si>
+  <si>
+    <t>Key</t>
+  </si>
+  <si>
+    <t>Address</t>
+  </si>
+  <si>
+    <t>ProductName</t>
+  </si>
+  <si>
+    <t>ProductCategory</t>
+  </si>
+  <si>
+    <t>ProductSubCategory</t>
+  </si>
+  <si>
+    <t>ProductPrice</t>
+  </si>
+  <si>
+    <t>ProductDescription</t>
+  </si>
+  <si>
+    <t>ProductFor</t>
+  </si>
+  <si>
+    <t>Country</t>
+  </si>
+  <si>
+    <t>qaclick123</t>
+  </si>
+  <si>
+    <t>Summer Walk, Africa</t>
   </si>
 </sst>
 </file>
@@ -157,10 +211,19 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -475,100 +538,246 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DF48170A-A807-4960-A9CB-7EA2270834B2}">
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:M8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="15" customWidth="1"/>
+    <col min="1" max="1" width="13.5703125" style="5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.7109375" style="5" customWidth="1"/>
+    <col min="3" max="3" width="7.5703125" style="5" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="6" style="5" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.140625" style="5" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.28515625" style="5" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="15.85546875" style="5" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="19.28515625" style="5" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="12.28515625" style="5" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="18.28515625" style="5" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="10.7109375" style="5" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="8" style="5" bestFit="1" customWidth="1"/>
+    <col min="14" max="16384" width="9.140625" style="5"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="2" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
+      <c r="E1" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="F1" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="G1" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="H1" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="I1" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="J1" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="K1" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="L1" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="M1" s="4" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A2" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="C2" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="D2" s="3" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
+      <c r="E2" s="3"/>
+      <c r="F2" s="3"/>
+      <c r="G2" s="3"/>
+      <c r="H2" s="3"/>
+      <c r="I2" s="3"/>
+      <c r="J2" s="3"/>
+      <c r="K2" s="3"/>
+      <c r="L2" s="3"/>
+      <c r="M2" s="3"/>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="B3" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="C3" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="D3" s="1" t="s">
+      <c r="D3" s="3" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" s="1" t="s">
+      <c r="E3" s="3"/>
+      <c r="F3" s="3"/>
+      <c r="G3" s="3"/>
+      <c r="H3" s="3"/>
+      <c r="I3" s="3"/>
+      <c r="J3" s="3"/>
+      <c r="K3" s="3"/>
+      <c r="L3" s="3"/>
+      <c r="M3" s="3"/>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="B4" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="C4" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="D4" s="1">
+      <c r="D4" s="3">
         <v>123</v>
       </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" s="1" t="s">
+      <c r="E4" s="3"/>
+      <c r="F4" s="3"/>
+      <c r="G4" s="3"/>
+      <c r="H4" s="3"/>
+      <c r="I4" s="3"/>
+      <c r="J4" s="3"/>
+      <c r="K4" s="3"/>
+      <c r="L4" s="3"/>
+      <c r="M4" s="3"/>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="B5" s="1">
+      <c r="B5" s="3">
         <v>234</v>
       </c>
-      <c r="C5" s="1">
+      <c r="C5" s="3">
         <v>567</v>
       </c>
-      <c r="D5" s="1">
+      <c r="D5" s="3">
         <v>899</v>
       </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" s="2" t="s">
+      <c r="E5" s="3"/>
+      <c r="F5" s="3"/>
+      <c r="G5" s="3"/>
+      <c r="H5" s="3"/>
+      <c r="I5" s="3"/>
+      <c r="J5" s="3"/>
+      <c r="K5" s="3"/>
+      <c r="L5" s="3"/>
+      <c r="M5" s="3"/>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A6" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B6" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="C6" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="D6" s="2" t="s">
+      <c r="D6" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="E6" s="2" t="s">
+      <c r="E6" s="4" t="s">
         <v>21</v>
+      </c>
+      <c r="F6" s="3"/>
+      <c r="G6" s="3"/>
+      <c r="H6" s="3"/>
+      <c r="I6" s="3"/>
+      <c r="J6" s="3"/>
+      <c r="K6" s="3"/>
+      <c r="L6" s="3"/>
+      <c r="M6" s="3"/>
+    </row>
+    <row r="7" spans="1:13" ht="60" x14ac:dyDescent="0.25">
+      <c r="A7" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="D7" s="3"/>
+      <c r="E7" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="G7" s="3"/>
+      <c r="H7" s="3"/>
+      <c r="I7" s="3"/>
+      <c r="J7" s="3"/>
+      <c r="K7" s="3"/>
+      <c r="L7" s="3"/>
+      <c r="M7" s="3"/>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A8" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="E8" s="3">
+        <v>11500</v>
+      </c>
+      <c r="F8" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="G8" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="H8" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="I8" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="J8" s="3">
+        <v>100</v>
+      </c>
+      <c r="K8" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="L8" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="M8" s="3" t="s">
+        <v>29</v>
       </c>
     </row>
   </sheetData>

</xml_diff>